<commit_message>
Add addresses and Apple/Google map links to practices, events and tournaments
- Events, single dates of a series and travel tournaments' hotels take a street address.
- Every place on the site becomes a map link: the address opens Apple Maps on
  Apple devices and Google Maps elsewhere, with a menu offering both. Without an
  address, the link searches for the venue and city.
- Calendar entries include the address; import reads Address and Hotel address columns.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011CHHr9uJweMf8dxpt7sEKV
</commit_message>
<xml_diff>
--- a/api/test/import/club-sample.xlsx
+++ b/api/test/import/club-sample.xlsx
@@ -448,6 +448,11 @@
         <t>Practice uniform color. New colors are added to the team's list.</t>
       </text>
     </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Street address. Families get a map link; without one the map searches the location.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -491,6 +496,16 @@
     <comment ref="V1" authorId="0" shapeId="0">
       <text>
         <t>Practices only.</t>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
+      <text>
+        <t>Street address of the venue. Families get a map link; without one the map searches the venue and city.</t>
+      </text>
+    </comment>
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <t>Travel tournaments: the team hotel's street address.</t>
       </text>
     </comment>
   </commentList>
@@ -10631,7 +10646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1000"/>
+  <dimension ref="A1:M1000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10646,6 +10661,7 @@
     <col width="9" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -10709,6 +10725,11 @@
           <t>Note</t>
         </is>
       </c>
+      <c r="M1" s="10" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
@@ -10765,6 +10786,11 @@
       <c r="L2" s="11" t="inlineStr">
         <is>
           <t>Bring both jerseys</t>
+        </is>
+      </c>
+      <c r="M2" s="11" t="inlineStr">
+        <is>
+          <t>1234 Example Rd, Roswell, GA 30076</t>
         </is>
       </c>
     </row>
@@ -10807,6 +10833,7 @@
       <c r="J3" s="6" t="inlineStr"/>
       <c r="K3" s="6" t="inlineStr"/>
       <c r="L3" s="6" t="inlineStr"/>
+      <c r="M3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -10859,6 +10886,7 @@
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr"/>
+      <c r="M4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n"/>
@@ -10873,6 +10901,7 @@
       <c r="J5" s="6" t="n"/>
       <c r="K5" s="6" t="n"/>
       <c r="L5" s="6" t="n"/>
+      <c r="M5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n"/>
@@ -10887,6 +10916,7 @@
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
       <c r="L6" s="6" t="n"/>
+      <c r="M6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n"/>
@@ -10901,6 +10931,7 @@
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="n"/>
       <c r="L7" s="6" t="n"/>
+      <c r="M7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n"/>
@@ -10915,6 +10946,7 @@
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="6" t="n"/>
+      <c r="M8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n"/>
@@ -10929,6 +10961,7 @@
       <c r="J9" s="6" t="n"/>
       <c r="K9" s="6" t="n"/>
       <c r="L9" s="6" t="n"/>
+      <c r="M9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
@@ -10943,6 +10976,7 @@
       <c r="J10" s="6" t="n"/>
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="6" t="n"/>
+      <c r="M10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>
@@ -10957,6 +10991,7 @@
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="6" t="n"/>
       <c r="L11" s="6" t="n"/>
+      <c r="M11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n"/>
@@ -10971,6 +11006,7 @@
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="6" t="n"/>
       <c r="L12" s="6" t="n"/>
+      <c r="M12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
@@ -10985,6 +11021,7 @@
       <c r="J13" s="6" t="n"/>
       <c r="K13" s="6" t="n"/>
       <c r="L13" s="6" t="n"/>
+      <c r="M13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
@@ -10999,6 +11036,7 @@
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
       <c r="L14" s="6" t="n"/>
+      <c r="M14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n"/>
@@ -11013,6 +11051,7 @@
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="6" t="n"/>
       <c r="L15" s="6" t="n"/>
+      <c r="M15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n"/>
@@ -11027,6 +11066,7 @@
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="6" t="n"/>
       <c r="L16" s="6" t="n"/>
+      <c r="M16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n"/>
@@ -11041,6 +11081,7 @@
       <c r="J17" s="6" t="n"/>
       <c r="K17" s="6" t="n"/>
       <c r="L17" s="6" t="n"/>
+      <c r="M17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
@@ -11055,6 +11096,7 @@
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="6" t="n"/>
       <c r="L18" s="6" t="n"/>
+      <c r="M18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n"/>
@@ -11069,6 +11111,7 @@
       <c r="J19" s="6" t="n"/>
       <c r="K19" s="6" t="n"/>
       <c r="L19" s="6" t="n"/>
+      <c r="M19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n"/>
@@ -11083,6 +11126,7 @@
       <c r="J20" s="6" t="n"/>
       <c r="K20" s="6" t="n"/>
       <c r="L20" s="6" t="n"/>
+      <c r="M20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n"/>
@@ -11097,6 +11141,7 @@
       <c r="J21" s="6" t="n"/>
       <c r="K21" s="6" t="n"/>
       <c r="L21" s="6" t="n"/>
+      <c r="M21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n"/>
@@ -11111,6 +11156,7 @@
       <c r="J22" s="6" t="n"/>
       <c r="K22" s="6" t="n"/>
       <c r="L22" s="6" t="n"/>
+      <c r="M22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n"/>
@@ -11125,6 +11171,7 @@
       <c r="J23" s="6" t="n"/>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="6" t="n"/>
+      <c r="M23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n"/>
@@ -11139,6 +11186,7 @@
       <c r="J24" s="6" t="n"/>
       <c r="K24" s="6" t="n"/>
       <c r="L24" s="6" t="n"/>
+      <c r="M24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n"/>
@@ -11153,6 +11201,7 @@
       <c r="J25" s="6" t="n"/>
       <c r="K25" s="6" t="n"/>
       <c r="L25" s="6" t="n"/>
+      <c r="M25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n"/>
@@ -11167,6 +11216,7 @@
       <c r="J26" s="6" t="n"/>
       <c r="K26" s="6" t="n"/>
       <c r="L26" s="6" t="n"/>
+      <c r="M26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n"/>
@@ -11181,6 +11231,7 @@
       <c r="J27" s="6" t="n"/>
       <c r="K27" s="6" t="n"/>
       <c r="L27" s="6" t="n"/>
+      <c r="M27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n"/>
@@ -11195,6 +11246,7 @@
       <c r="J28" s="6" t="n"/>
       <c r="K28" s="6" t="n"/>
       <c r="L28" s="6" t="n"/>
+      <c r="M28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n"/>
@@ -11209,6 +11261,7 @@
       <c r="J29" s="6" t="n"/>
       <c r="K29" s="6" t="n"/>
       <c r="L29" s="6" t="n"/>
+      <c r="M29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n"/>
@@ -11223,6 +11276,7 @@
       <c r="J30" s="6" t="n"/>
       <c r="K30" s="6" t="n"/>
       <c r="L30" s="6" t="n"/>
+      <c r="M30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n"/>
@@ -11237,6 +11291,7 @@
       <c r="J31" s="6" t="n"/>
       <c r="K31" s="6" t="n"/>
       <c r="L31" s="6" t="n"/>
+      <c r="M31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n"/>
@@ -11251,6 +11306,7 @@
       <c r="J32" s="6" t="n"/>
       <c r="K32" s="6" t="n"/>
       <c r="L32" s="6" t="n"/>
+      <c r="M32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n"/>
@@ -11265,6 +11321,7 @@
       <c r="J33" s="6" t="n"/>
       <c r="K33" s="6" t="n"/>
       <c r="L33" s="6" t="n"/>
+      <c r="M33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n"/>
@@ -11279,6 +11336,7 @@
       <c r="J34" s="6" t="n"/>
       <c r="K34" s="6" t="n"/>
       <c r="L34" s="6" t="n"/>
+      <c r="M34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n"/>
@@ -11293,6 +11351,7 @@
       <c r="J35" s="6" t="n"/>
       <c r="K35" s="6" t="n"/>
       <c r="L35" s="6" t="n"/>
+      <c r="M35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n"/>
@@ -11307,6 +11366,7 @@
       <c r="J36" s="6" t="n"/>
       <c r="K36" s="6" t="n"/>
       <c r="L36" s="6" t="n"/>
+      <c r="M36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n"/>
@@ -11321,6 +11381,7 @@
       <c r="J37" s="6" t="n"/>
       <c r="K37" s="6" t="n"/>
       <c r="L37" s="6" t="n"/>
+      <c r="M37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n"/>
@@ -11335,6 +11396,7 @@
       <c r="J38" s="6" t="n"/>
       <c r="K38" s="6" t="n"/>
       <c r="L38" s="6" t="n"/>
+      <c r="M38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n"/>
@@ -11349,6 +11411,7 @@
       <c r="J39" s="6" t="n"/>
       <c r="K39" s="6" t="n"/>
       <c r="L39" s="6" t="n"/>
+      <c r="M39" s="6" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n"/>
@@ -11363,6 +11426,7 @@
       <c r="J40" s="6" t="n"/>
       <c r="K40" s="6" t="n"/>
       <c r="L40" s="6" t="n"/>
+      <c r="M40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n"/>
@@ -11377,6 +11441,7 @@
       <c r="J41" s="6" t="n"/>
       <c r="K41" s="6" t="n"/>
       <c r="L41" s="6" t="n"/>
+      <c r="M41" s="6" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n"/>
@@ -11391,6 +11456,7 @@
       <c r="J42" s="6" t="n"/>
       <c r="K42" s="6" t="n"/>
       <c r="L42" s="6" t="n"/>
+      <c r="M42" s="6" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n"/>
@@ -11405,6 +11471,7 @@
       <c r="J43" s="6" t="n"/>
       <c r="K43" s="6" t="n"/>
       <c r="L43" s="6" t="n"/>
+      <c r="M43" s="6" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n"/>
@@ -11419,6 +11486,7 @@
       <c r="J44" s="6" t="n"/>
       <c r="K44" s="6" t="n"/>
       <c r="L44" s="6" t="n"/>
+      <c r="M44" s="6" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n"/>
@@ -11433,6 +11501,7 @@
       <c r="J45" s="6" t="n"/>
       <c r="K45" s="6" t="n"/>
       <c r="L45" s="6" t="n"/>
+      <c r="M45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n"/>
@@ -11447,6 +11516,7 @@
       <c r="J46" s="6" t="n"/>
       <c r="K46" s="6" t="n"/>
       <c r="L46" s="6" t="n"/>
+      <c r="M46" s="6" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n"/>
@@ -11461,6 +11531,7 @@
       <c r="J47" s="6" t="n"/>
       <c r="K47" s="6" t="n"/>
       <c r="L47" s="6" t="n"/>
+      <c r="M47" s="6" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="n"/>
@@ -11475,6 +11546,7 @@
       <c r="J48" s="6" t="n"/>
       <c r="K48" s="6" t="n"/>
       <c r="L48" s="6" t="n"/>
+      <c r="M48" s="6" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="6" t="n"/>
@@ -11489,6 +11561,7 @@
       <c r="J49" s="6" t="n"/>
       <c r="K49" s="6" t="n"/>
       <c r="L49" s="6" t="n"/>
+      <c r="M49" s="6" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="6" t="n"/>
@@ -11503,6 +11576,7 @@
       <c r="J50" s="6" t="n"/>
       <c r="K50" s="6" t="n"/>
       <c r="L50" s="6" t="n"/>
+      <c r="M50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="n"/>
@@ -11517,6 +11591,7 @@
       <c r="J51" s="6" t="n"/>
       <c r="K51" s="6" t="n"/>
       <c r="L51" s="6" t="n"/>
+      <c r="M51" s="6" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n"/>
@@ -11531,6 +11606,7 @@
       <c r="J52" s="6" t="n"/>
       <c r="K52" s="6" t="n"/>
       <c r="L52" s="6" t="n"/>
+      <c r="M52" s="6" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="n"/>
@@ -11545,6 +11621,7 @@
       <c r="J53" s="6" t="n"/>
       <c r="K53" s="6" t="n"/>
       <c r="L53" s="6" t="n"/>
+      <c r="M53" s="6" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="n"/>
@@ -11559,6 +11636,7 @@
       <c r="J54" s="6" t="n"/>
       <c r="K54" s="6" t="n"/>
       <c r="L54" s="6" t="n"/>
+      <c r="M54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="n"/>
@@ -11573,6 +11651,7 @@
       <c r="J55" s="6" t="n"/>
       <c r="K55" s="6" t="n"/>
       <c r="L55" s="6" t="n"/>
+      <c r="M55" s="6" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="6" t="n"/>
@@ -11587,6 +11666,7 @@
       <c r="J56" s="6" t="n"/>
       <c r="K56" s="6" t="n"/>
       <c r="L56" s="6" t="n"/>
+      <c r="M56" s="6" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="6" t="n"/>
@@ -11601,6 +11681,7 @@
       <c r="J57" s="6" t="n"/>
       <c r="K57" s="6" t="n"/>
       <c r="L57" s="6" t="n"/>
+      <c r="M57" s="6" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="n"/>
@@ -11615,6 +11696,7 @@
       <c r="J58" s="6" t="n"/>
       <c r="K58" s="6" t="n"/>
       <c r="L58" s="6" t="n"/>
+      <c r="M58" s="6" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="6" t="n"/>
@@ -11629,6 +11711,7 @@
       <c r="J59" s="6" t="n"/>
       <c r="K59" s="6" t="n"/>
       <c r="L59" s="6" t="n"/>
+      <c r="M59" s="6" t="n"/>
     </row>
     <row r="60">
       <c r="F60" s="24" t="n"/>
@@ -15423,7 +15506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V1000"/>
+  <dimension ref="A1:X1000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15448,6 +15531,8 @@
     <col width="36" customWidth="1" min="20" max="20"/>
     <col width="9" customWidth="1" min="21" max="21"/>
     <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="30" customWidth="1" min="23" max="23"/>
+    <col width="30" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -15559,6 +15644,16 @@
       <c r="V1" s="10" t="inlineStr">
         <is>
           <t>Uniform color</t>
+        </is>
+      </c>
+      <c r="W1" s="10" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="X1" s="10" t="inlineStr">
+        <is>
+          <t>Hotel address</t>
         </is>
       </c>
     </row>
@@ -15633,6 +15728,12 @@
       </c>
       <c r="U2" s="11" t="inlineStr"/>
       <c r="V2" s="11" t="inlineStr"/>
+      <c r="W2" s="11" t="inlineStr">
+        <is>
+          <t>285 Andrew Young International Blvd NW, Atlanta, GA 30313</t>
+        </is>
+      </c>
+      <c r="X2" s="11" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -15703,6 +15804,8 @@
       <c r="T3" s="6" t="inlineStr"/>
       <c r="U3" s="6" t="n"/>
       <c r="V3" s="6" t="n"/>
+      <c r="W3" s="6" t="n"/>
+      <c r="X3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -15741,6 +15844,8 @@
       <c r="T4" s="6" t="inlineStr"/>
       <c r="U4" s="6" t="n"/>
       <c r="V4" s="6" t="n"/>
+      <c r="W4" s="6" t="n"/>
+      <c r="X4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n"/>
@@ -15765,6 +15870,8 @@
       <c r="T5" s="6" t="n"/>
       <c r="U5" s="6" t="n"/>
       <c r="V5" s="6" t="n"/>
+      <c r="W5" s="6" t="n"/>
+      <c r="X5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n"/>
@@ -15789,6 +15896,8 @@
       <c r="T6" s="6" t="n"/>
       <c r="U6" s="6" t="n"/>
       <c r="V6" s="6" t="n"/>
+      <c r="W6" s="6" t="n"/>
+      <c r="X6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n"/>
@@ -15813,6 +15922,8 @@
       <c r="T7" s="6" t="n"/>
       <c r="U7" s="6" t="n"/>
       <c r="V7" s="6" t="n"/>
+      <c r="W7" s="6" t="n"/>
+      <c r="X7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n"/>
@@ -15837,6 +15948,8 @@
       <c r="T8" s="6" t="n"/>
       <c r="U8" s="6" t="n"/>
       <c r="V8" s="6" t="n"/>
+      <c r="W8" s="6" t="n"/>
+      <c r="X8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n"/>
@@ -15861,6 +15974,8 @@
       <c r="T9" s="6" t="n"/>
       <c r="U9" s="6" t="n"/>
       <c r="V9" s="6" t="n"/>
+      <c r="W9" s="6" t="n"/>
+      <c r="X9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
@@ -15885,6 +16000,8 @@
       <c r="T10" s="6" t="n"/>
       <c r="U10" s="6" t="n"/>
       <c r="V10" s="6" t="n"/>
+      <c r="W10" s="6" t="n"/>
+      <c r="X10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>
@@ -15909,6 +16026,8 @@
       <c r="T11" s="6" t="n"/>
       <c r="U11" s="6" t="n"/>
       <c r="V11" s="6" t="n"/>
+      <c r="W11" s="6" t="n"/>
+      <c r="X11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n"/>
@@ -15933,6 +16052,8 @@
       <c r="T12" s="6" t="n"/>
       <c r="U12" s="6" t="n"/>
       <c r="V12" s="6" t="n"/>
+      <c r="W12" s="6" t="n"/>
+      <c r="X12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
@@ -15957,6 +16078,8 @@
       <c r="T13" s="6" t="n"/>
       <c r="U13" s="6" t="n"/>
       <c r="V13" s="6" t="n"/>
+      <c r="W13" s="6" t="n"/>
+      <c r="X13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
@@ -15981,6 +16104,8 @@
       <c r="T14" s="6" t="n"/>
       <c r="U14" s="6" t="n"/>
       <c r="V14" s="6" t="n"/>
+      <c r="W14" s="6" t="n"/>
+      <c r="X14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n"/>
@@ -16005,6 +16130,8 @@
       <c r="T15" s="6" t="n"/>
       <c r="U15" s="6" t="n"/>
       <c r="V15" s="6" t="n"/>
+      <c r="W15" s="6" t="n"/>
+      <c r="X15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n"/>
@@ -16029,6 +16156,8 @@
       <c r="T16" s="6" t="n"/>
       <c r="U16" s="6" t="n"/>
       <c r="V16" s="6" t="n"/>
+      <c r="W16" s="6" t="n"/>
+      <c r="X16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n"/>
@@ -16053,6 +16182,8 @@
       <c r="T17" s="6" t="n"/>
       <c r="U17" s="6" t="n"/>
       <c r="V17" s="6" t="n"/>
+      <c r="W17" s="6" t="n"/>
+      <c r="X17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
@@ -16077,6 +16208,8 @@
       <c r="T18" s="6" t="n"/>
       <c r="U18" s="6" t="n"/>
       <c r="V18" s="6" t="n"/>
+      <c r="W18" s="6" t="n"/>
+      <c r="X18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n"/>
@@ -16101,6 +16234,8 @@
       <c r="T19" s="6" t="n"/>
       <c r="U19" s="6" t="n"/>
       <c r="V19" s="6" t="n"/>
+      <c r="W19" s="6" t="n"/>
+      <c r="X19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n"/>
@@ -16125,6 +16260,8 @@
       <c r="T20" s="6" t="n"/>
       <c r="U20" s="6" t="n"/>
       <c r="V20" s="6" t="n"/>
+      <c r="W20" s="6" t="n"/>
+      <c r="X20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n"/>
@@ -16149,6 +16286,8 @@
       <c r="T21" s="6" t="n"/>
       <c r="U21" s="6" t="n"/>
       <c r="V21" s="6" t="n"/>
+      <c r="W21" s="6" t="n"/>
+      <c r="X21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n"/>
@@ -16173,6 +16312,8 @@
       <c r="T22" s="6" t="n"/>
       <c r="U22" s="6" t="n"/>
       <c r="V22" s="6" t="n"/>
+      <c r="W22" s="6" t="n"/>
+      <c r="X22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n"/>
@@ -16197,6 +16338,8 @@
       <c r="T23" s="6" t="n"/>
       <c r="U23" s="6" t="n"/>
       <c r="V23" s="6" t="n"/>
+      <c r="W23" s="6" t="n"/>
+      <c r="X23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n"/>
@@ -16221,6 +16364,8 @@
       <c r="T24" s="6" t="n"/>
       <c r="U24" s="6" t="n"/>
       <c r="V24" s="6" t="n"/>
+      <c r="W24" s="6" t="n"/>
+      <c r="X24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n"/>
@@ -16245,6 +16390,8 @@
       <c r="T25" s="6" t="n"/>
       <c r="U25" s="6" t="n"/>
       <c r="V25" s="6" t="n"/>
+      <c r="W25" s="6" t="n"/>
+      <c r="X25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n"/>
@@ -16269,6 +16416,8 @@
       <c r="T26" s="6" t="n"/>
       <c r="U26" s="6" t="n"/>
       <c r="V26" s="6" t="n"/>
+      <c r="W26" s="6" t="n"/>
+      <c r="X26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n"/>
@@ -16293,6 +16442,8 @@
       <c r="T27" s="6" t="n"/>
       <c r="U27" s="6" t="n"/>
       <c r="V27" s="6" t="n"/>
+      <c r="W27" s="6" t="n"/>
+      <c r="X27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n"/>
@@ -16317,6 +16468,8 @@
       <c r="T28" s="6" t="n"/>
       <c r="U28" s="6" t="n"/>
       <c r="V28" s="6" t="n"/>
+      <c r="W28" s="6" t="n"/>
+      <c r="X28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n"/>
@@ -16341,6 +16494,8 @@
       <c r="T29" s="6" t="n"/>
       <c r="U29" s="6" t="n"/>
       <c r="V29" s="6" t="n"/>
+      <c r="W29" s="6" t="n"/>
+      <c r="X29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n"/>
@@ -16365,6 +16520,8 @@
       <c r="T30" s="6" t="n"/>
       <c r="U30" s="6" t="n"/>
       <c r="V30" s="6" t="n"/>
+      <c r="W30" s="6" t="n"/>
+      <c r="X30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n"/>
@@ -16389,6 +16546,8 @@
       <c r="T31" s="6" t="n"/>
       <c r="U31" s="6" t="n"/>
       <c r="V31" s="6" t="n"/>
+      <c r="W31" s="6" t="n"/>
+      <c r="X31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n"/>
@@ -16413,6 +16572,8 @@
       <c r="T32" s="6" t="n"/>
       <c r="U32" s="6" t="n"/>
       <c r="V32" s="6" t="n"/>
+      <c r="W32" s="6" t="n"/>
+      <c r="X32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n"/>
@@ -16437,6 +16598,8 @@
       <c r="T33" s="6" t="n"/>
       <c r="U33" s="6" t="n"/>
       <c r="V33" s="6" t="n"/>
+      <c r="W33" s="6" t="n"/>
+      <c r="X33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n"/>
@@ -16461,6 +16624,8 @@
       <c r="T34" s="6" t="n"/>
       <c r="U34" s="6" t="n"/>
       <c r="V34" s="6" t="n"/>
+      <c r="W34" s="6" t="n"/>
+      <c r="X34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n"/>
@@ -16485,6 +16650,8 @@
       <c r="T35" s="6" t="n"/>
       <c r="U35" s="6" t="n"/>
       <c r="V35" s="6" t="n"/>
+      <c r="W35" s="6" t="n"/>
+      <c r="X35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n"/>
@@ -16509,6 +16676,8 @@
       <c r="T36" s="6" t="n"/>
       <c r="U36" s="6" t="n"/>
       <c r="V36" s="6" t="n"/>
+      <c r="W36" s="6" t="n"/>
+      <c r="X36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n"/>
@@ -16533,6 +16702,8 @@
       <c r="T37" s="6" t="n"/>
       <c r="U37" s="6" t="n"/>
       <c r="V37" s="6" t="n"/>
+      <c r="W37" s="6" t="n"/>
+      <c r="X37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n"/>
@@ -16557,6 +16728,8 @@
       <c r="T38" s="6" t="n"/>
       <c r="U38" s="6" t="n"/>
       <c r="V38" s="6" t="n"/>
+      <c r="W38" s="6" t="n"/>
+      <c r="X38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n"/>
@@ -16581,6 +16754,8 @@
       <c r="T39" s="6" t="n"/>
       <c r="U39" s="6" t="n"/>
       <c r="V39" s="6" t="n"/>
+      <c r="W39" s="6" t="n"/>
+      <c r="X39" s="6" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n"/>
@@ -16605,6 +16780,8 @@
       <c r="T40" s="6" t="n"/>
       <c r="U40" s="6" t="n"/>
       <c r="V40" s="6" t="n"/>
+      <c r="W40" s="6" t="n"/>
+      <c r="X40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n"/>
@@ -16629,6 +16806,8 @@
       <c r="T41" s="6" t="n"/>
       <c r="U41" s="6" t="n"/>
       <c r="V41" s="6" t="n"/>
+      <c r="W41" s="6" t="n"/>
+      <c r="X41" s="6" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n"/>
@@ -16653,6 +16832,8 @@
       <c r="T42" s="6" t="n"/>
       <c r="U42" s="6" t="n"/>
       <c r="V42" s="6" t="n"/>
+      <c r="W42" s="6" t="n"/>
+      <c r="X42" s="6" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n"/>
@@ -16677,6 +16858,8 @@
       <c r="T43" s="6" t="n"/>
       <c r="U43" s="6" t="n"/>
       <c r="V43" s="6" t="n"/>
+      <c r="W43" s="6" t="n"/>
+      <c r="X43" s="6" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n"/>
@@ -16701,6 +16884,8 @@
       <c r="T44" s="6" t="n"/>
       <c r="U44" s="6" t="n"/>
       <c r="V44" s="6" t="n"/>
+      <c r="W44" s="6" t="n"/>
+      <c r="X44" s="6" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n"/>
@@ -16725,6 +16910,8 @@
       <c r="T45" s="6" t="n"/>
       <c r="U45" s="6" t="n"/>
       <c r="V45" s="6" t="n"/>
+      <c r="W45" s="6" t="n"/>
+      <c r="X45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n"/>
@@ -16749,6 +16936,8 @@
       <c r="T46" s="6" t="n"/>
       <c r="U46" s="6" t="n"/>
       <c r="V46" s="6" t="n"/>
+      <c r="W46" s="6" t="n"/>
+      <c r="X46" s="6" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n"/>
@@ -16773,6 +16962,8 @@
       <c r="T47" s="6" t="n"/>
       <c r="U47" s="6" t="n"/>
       <c r="V47" s="6" t="n"/>
+      <c r="W47" s="6" t="n"/>
+      <c r="X47" s="6" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="n"/>
@@ -16797,6 +16988,8 @@
       <c r="T48" s="6" t="n"/>
       <c r="U48" s="6" t="n"/>
       <c r="V48" s="6" t="n"/>
+      <c r="W48" s="6" t="n"/>
+      <c r="X48" s="6" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="6" t="n"/>
@@ -16821,6 +17014,8 @@
       <c r="T49" s="6" t="n"/>
       <c r="U49" s="6" t="n"/>
       <c r="V49" s="6" t="n"/>
+      <c r="W49" s="6" t="n"/>
+      <c r="X49" s="6" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="6" t="n"/>
@@ -16845,6 +17040,8 @@
       <c r="T50" s="6" t="n"/>
       <c r="U50" s="6" t="n"/>
       <c r="V50" s="6" t="n"/>
+      <c r="W50" s="6" t="n"/>
+      <c r="X50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="n"/>
@@ -16869,6 +17066,8 @@
       <c r="T51" s="6" t="n"/>
       <c r="U51" s="6" t="n"/>
       <c r="V51" s="6" t="n"/>
+      <c r="W51" s="6" t="n"/>
+      <c r="X51" s="6" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n"/>
@@ -16893,6 +17092,8 @@
       <c r="T52" s="6" t="n"/>
       <c r="U52" s="6" t="n"/>
       <c r="V52" s="6" t="n"/>
+      <c r="W52" s="6" t="n"/>
+      <c r="X52" s="6" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="n"/>
@@ -16917,6 +17118,8 @@
       <c r="T53" s="6" t="n"/>
       <c r="U53" s="6" t="n"/>
       <c r="V53" s="6" t="n"/>
+      <c r="W53" s="6" t="n"/>
+      <c r="X53" s="6" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="n"/>
@@ -16941,6 +17144,8 @@
       <c r="T54" s="6" t="n"/>
       <c r="U54" s="6" t="n"/>
       <c r="V54" s="6" t="n"/>
+      <c r="W54" s="6" t="n"/>
+      <c r="X54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="n"/>
@@ -16965,6 +17170,8 @@
       <c r="T55" s="6" t="n"/>
       <c r="U55" s="6" t="n"/>
       <c r="V55" s="6" t="n"/>
+      <c r="W55" s="6" t="n"/>
+      <c r="X55" s="6" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="6" t="n"/>
@@ -16989,6 +17196,8 @@
       <c r="T56" s="6" t="n"/>
       <c r="U56" s="6" t="n"/>
       <c r="V56" s="6" t="n"/>
+      <c r="W56" s="6" t="n"/>
+      <c r="X56" s="6" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="6" t="n"/>
@@ -17013,6 +17222,8 @@
       <c r="T57" s="6" t="n"/>
       <c r="U57" s="6" t="n"/>
       <c r="V57" s="6" t="n"/>
+      <c r="W57" s="6" t="n"/>
+      <c r="X57" s="6" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="n"/>
@@ -17037,6 +17248,8 @@
       <c r="T58" s="6" t="n"/>
       <c r="U58" s="6" t="n"/>
       <c r="V58" s="6" t="n"/>
+      <c r="W58" s="6" t="n"/>
+      <c r="X58" s="6" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="6" t="n"/>
@@ -17061,6 +17274,8 @@
       <c r="T59" s="6" t="n"/>
       <c r="U59" s="6" t="n"/>
       <c r="V59" s="6" t="n"/>
+      <c r="W59" s="6" t="n"/>
+      <c r="X59" s="6" t="n"/>
     </row>
     <row r="60">
       <c r="D60" s="24" t="n"/>

</xml_diff>